<commit_message>
Fully translate AI-DQA English DFMEA templates to remove all Chinese labels.
Rebuild Template-1/Template-2 from Chinese shells with comprehensive header translation, clear example data, English sheet tab names, and DFMEA Standard Form sheet alias support.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/Template-1-DFMEA-Legacy.xlsx
+++ b/templates/Template-1-DFMEA-Legacy.xlsx
@@ -1013,7 +1013,7 @@
     <row r="2" ht="21" customHeight="1" s="80">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>(DFMEA)</t>
+          <t>（DFMEA)</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       <c r="A4" s="26" t="n"/>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>子System</t>
+          <t>Subsystem</t>
         </is>
       </c>
       <c r="C4" s="27" t="n"/>
@@ -1061,7 +1061,7 @@
       <c r="L4" s="28" t="n"/>
       <c r="M4" s="28" t="inlineStr">
         <is>
-          <t>FMEA编号</t>
+          <t>FMEA no.</t>
         </is>
       </c>
       <c r="N4" s="39" t="n"/>
@@ -1084,7 +1084,7 @@
       <c r="F5" s="81" t="n"/>
       <c r="G5" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">            Design Responsibility</t>
+          <t xml:space="preserve">            Design responsibility</t>
         </is>
       </c>
       <c r="H5" s="54" t="n"/>
@@ -1094,12 +1094,12 @@
       <c r="L5" s="43" t="n"/>
       <c r="M5" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">第  1 页 </t>
+          <t xml:space="preserve">Page </t>
         </is>
       </c>
       <c r="N5" s="27" t="inlineStr">
         <is>
-          <t xml:space="preserve">   共   页</t>
+          <t xml:space="preserve">   of</t>
         </is>
       </c>
       <c r="O5" s="27" t="n"/>
@@ -1111,7 +1111,7 @@
     <row r="6" ht="18" customHeight="1" s="80">
       <c r="A6" s="31" t="inlineStr">
         <is>
-          <t>Model / Project</t>
+          <t>Model / project</t>
         </is>
       </c>
       <c r="B6" s="32" t="n"/>
@@ -1121,7 +1121,7 @@
       <c r="F6" s="81" t="n"/>
       <c r="G6" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">            Key Date</t>
+          <t xml:space="preserve">            Key date</t>
         </is>
       </c>
       <c r="H6" s="55" t="n"/>
@@ -1131,7 +1131,7 @@
       <c r="L6" s="44" t="n"/>
       <c r="M6" s="44" t="inlineStr">
         <is>
-          <t>编 制 人</t>
+          <t>Prepared by</t>
         </is>
       </c>
       <c r="N6" s="47" t="n"/>
@@ -1144,7 +1144,7 @@
     <row r="7" ht="16.5" customHeight="1" s="80">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Core Team     　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
+          <t xml:space="preserve">Core team     　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
         </is>
       </c>
       <c r="B7" s="53" t="n"/>
@@ -1160,7 +1160,7 @@
       <c r="L7" s="42" t="n"/>
       <c r="M7" s="79" t="inlineStr">
         <is>
-          <t>FMEA日期（编制）</t>
+          <t>FMEA date (original)</t>
         </is>
       </c>
       <c r="O7" s="79" t="n"/>
@@ -1199,32 +1199,32 @@
       </c>
       <c r="C9" s="65" t="inlineStr">
         <is>
-          <t>Potential Failure Mode</t>
+          <t>Potential failure mode</t>
         </is>
       </c>
       <c r="D9" s="65" t="inlineStr">
         <is>
-          <t>潜在失效   　后果</t>
+          <t>Potential failure effect</t>
         </is>
       </c>
       <c r="E9" s="65" t="inlineStr">
         <is>
-          <t>严  重 度  S</t>
+          <t>Severity (S)</t>
         </is>
       </c>
       <c r="F9" s="65" t="inlineStr">
         <is>
-          <t>特殊特性</t>
+          <t>Special characteristics</t>
         </is>
       </c>
       <c r="G9" s="65" t="inlineStr">
         <is>
-          <t>潜在失效起因/机理</t>
+          <t>Potential failure cause / mechanism</t>
         </is>
       </c>
       <c r="H9" s="65" t="inlineStr">
         <is>
-          <t>现行过程</t>
+          <t>Current process</t>
         </is>
       </c>
       <c r="I9" s="82" t="n"/>
@@ -1233,17 +1233,17 @@
       <c r="L9" s="83" t="n"/>
       <c r="M9" s="65" t="inlineStr">
         <is>
-          <t>建  议　　 措  施</t>
+          <t>Recommended actions</t>
         </is>
       </c>
       <c r="N9" s="65" t="inlineStr">
         <is>
-          <t>责任及目标 完成日期</t>
+          <t>Responsibility &amp; target completion date</t>
         </is>
       </c>
       <c r="O9" s="36" t="inlineStr">
         <is>
-          <t>措  施  结  果</t>
+          <t>Action results</t>
         </is>
       </c>
       <c r="P9" s="84" t="n"/>
@@ -1261,54 +1261,54 @@
       <c r="G10" s="86" t="n"/>
       <c r="H10" s="36" t="inlineStr">
         <is>
-          <t>频 数  O</t>
+          <t>Occurrence (O)</t>
         </is>
       </c>
       <c r="I10" s="36" t="inlineStr">
         <is>
-          <t>控制Prevention</t>
+          <t>Prevention control</t>
         </is>
       </c>
       <c r="J10" s="36" t="inlineStr">
         <is>
-          <t>控制Detection</t>
+          <t>Detection control</t>
         </is>
       </c>
       <c r="K10" s="36" t="inlineStr">
         <is>
-          <t>探 测 度  D</t>
+          <t>Detection (D)</t>
         </is>
       </c>
       <c r="L10" s="38" t="inlineStr">
         <is>
-          <t>风　险　顺　序　数RPN</t>
+          <t>RPN</t>
         </is>
       </c>
       <c r="M10" s="86" t="n"/>
       <c r="N10" s="86" t="n"/>
       <c r="O10" s="65" t="inlineStr">
         <is>
-          <t>采取的　  措  施</t>
+          <t>Actions taken</t>
         </is>
       </c>
       <c r="P10" s="65" t="inlineStr">
         <is>
-          <t>严　重　度　 S</t>
+          <t>Severity (S)</t>
         </is>
       </c>
       <c r="Q10" s="65" t="inlineStr">
         <is>
-          <t>频　度　O</t>
+          <t>Occurrence (O)</t>
         </is>
       </c>
       <c r="R10" s="65" t="inlineStr">
         <is>
-          <t>探　测　度　D</t>
+          <t>Detection (D)</t>
         </is>
       </c>
       <c r="S10" s="65" t="inlineStr">
         <is>
-          <t>风　险　顺　序　数RPN</t>
+          <t>RPN</t>
         </is>
       </c>
     </row>
@@ -1973,13 +1973,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R16"/>
+  <dimension ref="A1:AD16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>表单编号：</t>
+          <t>Form no.:</t>
         </is>
       </c>
       <c r="B1" s="4" t="n"/>
@@ -2007,7 +2007,7 @@
       <c r="F2" s="16" t="n"/>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   （设计 FMEA）                         </t>
+          <t xml:space="preserve">   (Design FMEA)                         </t>
         </is>
       </c>
       <c r="H2" s="4" t="n"/>
@@ -2037,7 +2037,7 @@
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>FMEA编号</t>
+          <t>FMEA no.</t>
         </is>
       </c>
       <c r="N3" s="17" t="n"/>
@@ -2047,41 +2047,17 @@
       <c r="R3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       产品名称：</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>壁挂式温湿度显示仪</t>
-        </is>
-      </c>
+      <c r="A4" s="69" t="n"/>
+      <c r="C4" s="7" t="n"/>
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="69" t="n"/>
       <c r="F4" s="16" t="n"/>
-      <c r="G4" s="70" t="inlineStr">
-        <is>
-          <t>Design Responsibility</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>李宁子</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>邱国财</t>
-        </is>
-      </c>
+      <c r="G4" s="70" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
-      <c r="M4" s="16" t="inlineStr">
-        <is>
-          <t>第  1 页    共   页</t>
-        </is>
-      </c>
+      <c r="M4" s="16" t="n"/>
       <c r="N4" s="16" t="n"/>
       <c r="O4" s="8" t="n"/>
       <c r="P4" s="8" t="n"/>
@@ -2089,54 +2065,26 @@
       <c r="R4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">       型号：</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>AS106</t>
-        </is>
-      </c>
+      <c r="A5" s="69" t="n"/>
+      <c r="C5" s="7" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="9" t="n"/>
       <c r="F5" s="16" t="n"/>
-      <c r="G5" s="70" t="inlineStr">
-        <is>
-          <t>Key Date</t>
-        </is>
-      </c>
+      <c r="G5" s="70" t="n"/>
       <c r="I5" s="19" t="n"/>
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
-      <c r="M5" s="69" t="inlineStr">
-        <is>
-          <t>编 制 人</t>
-        </is>
-      </c>
-      <c r="N5" s="12" t="inlineStr">
-        <is>
-          <t>丁和轩</t>
-        </is>
-      </c>
+      <c r="M5" s="69" t="n"/>
+      <c r="N5" s="12" t="n"/>
       <c r="O5" s="8" t="n"/>
       <c r="P5" s="8" t="n"/>
       <c r="Q5" s="8" t="n"/>
       <c r="R5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Core Team     　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　　</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>多功能小组</t>
-        </is>
-      </c>
+      <c r="A6" s="16" t="n"/>
+      <c r="B6" s="10" t="n"/>
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="12" t="n"/>
       <c r="E6" s="11" t="n"/>
@@ -2147,16 +2095,8 @@
       <c r="J6" s="12" t="n"/>
       <c r="K6" s="12" t="n"/>
       <c r="L6" s="16" t="n"/>
-      <c r="M6" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FMEA日期（编制）　　　</t>
-        </is>
-      </c>
-      <c r="P6" s="16" t="inlineStr">
-        <is>
-          <t>修订</t>
-        </is>
-      </c>
+      <c r="M6" s="69" t="n"/>
+      <c r="P6" s="16" t="n"/>
       <c r="Q6" s="16" t="n"/>
       <c r="R6" s="16" t="n"/>
     </row>
@@ -2181,76 +2121,20 @@
       <c r="R7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">　</t>
-        </is>
-      </c>
-      <c r="B8" s="77" t="inlineStr">
-        <is>
-          <t>潜在失效     模式</t>
-        </is>
-      </c>
-      <c r="C8" s="77" t="inlineStr">
-        <is>
-          <t>潜在失效   　后果</t>
-        </is>
-      </c>
-      <c r="D8" s="77" t="inlineStr">
-        <is>
-          <t>严  重 度  S</t>
-        </is>
-      </c>
-      <c r="E8" s="77" t="inlineStr">
-        <is>
-          <t>级 别</t>
-        </is>
-      </c>
-      <c r="F8" s="77" t="inlineStr">
-        <is>
-          <t>潜在失效     起因/机理</t>
-        </is>
-      </c>
-      <c r="G8" s="77" t="inlineStr">
-        <is>
-          <t>频 数  O</t>
-        </is>
-      </c>
-      <c r="H8" s="77" t="inlineStr">
-        <is>
-          <t>现行设计     控制Prevention</t>
-        </is>
-      </c>
-      <c r="I8" s="77" t="inlineStr">
-        <is>
-          <t>现行设计     控制Detection</t>
-        </is>
-      </c>
-      <c r="J8" s="77" t="inlineStr">
-        <is>
-          <t>探 测 度  D</t>
-        </is>
-      </c>
-      <c r="K8" s="77" t="inlineStr">
-        <is>
-          <t>风　险　顺　序　数RPN</t>
-        </is>
-      </c>
-      <c r="L8" s="77" t="inlineStr">
-        <is>
-          <t>建  议　　 措  施</t>
-        </is>
-      </c>
-      <c r="M8" s="77" t="inlineStr">
-        <is>
-          <t>责任及目标 完成日期</t>
-        </is>
-      </c>
-      <c r="N8" s="15" t="inlineStr">
-        <is>
-          <t>措  施  结  果</t>
-        </is>
-      </c>
+      <c r="A8" s="74" t="n"/>
+      <c r="B8" s="77" t="n"/>
+      <c r="C8" s="77" t="n"/>
+      <c r="D8" s="77" t="n"/>
+      <c r="E8" s="77" t="n"/>
+      <c r="F8" s="77" t="n"/>
+      <c r="G8" s="77" t="n"/>
+      <c r="H8" s="77" t="n"/>
+      <c r="I8" s="77" t="n"/>
+      <c r="J8" s="77" t="n"/>
+      <c r="K8" s="77" t="n"/>
+      <c r="L8" s="77" t="n"/>
+      <c r="M8" s="77" t="n"/>
+      <c r="N8" s="15" t="n"/>
       <c r="O8" s="84" t="n"/>
       <c r="P8" s="84" t="n"/>
       <c r="Q8" s="84" t="n"/>
@@ -2270,80 +2154,26 @@
       <c r="K9" s="86" t="n"/>
       <c r="L9" s="86" t="n"/>
       <c r="M9" s="86" t="n"/>
-      <c r="N9" s="77" t="inlineStr">
-        <is>
-          <t>采取的　  措  施</t>
-        </is>
-      </c>
-      <c r="O9" s="77" t="inlineStr">
-        <is>
-          <t>严　重　度　 S</t>
-        </is>
-      </c>
-      <c r="P9" s="77" t="inlineStr">
-        <is>
-          <t>频　度　O</t>
-        </is>
-      </c>
-      <c r="Q9" s="77" t="inlineStr">
-        <is>
-          <t>探　测　度　D</t>
-        </is>
-      </c>
-      <c r="R9" s="77" t="inlineStr">
-        <is>
-          <t>风　险　顺　序　数RPN</t>
-        </is>
-      </c>
+      <c r="N9" s="77" t="n"/>
+      <c r="O9" s="77" t="n"/>
+      <c r="P9" s="77" t="n"/>
+      <c r="Q9" s="77" t="n"/>
+      <c r="R9" s="77" t="n"/>
     </row>
     <row r="10" ht="132" customHeight="1" s="80">
       <c r="A10" s="76" t="n"/>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>气体的相对湿度在不同温度环境下一致性差。容易受外部高温电子元器件影响</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>相对湿度测量精度下降</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>气体的相对湿度，在很大程度上依赖于温度。故采样相对湿度时候要尽可能与环境温度一致。</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>设计电路时候远离热源</t>
-        </is>
-      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="14" t="n"/>
       <c r="I10" s="14" t="n"/>
-      <c r="J10" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="15" t="n">
-        <v>112</v>
-      </c>
-      <c r="L10" s="14" t="inlineStr">
-        <is>
-          <t>设计电路时候远离热源</t>
-        </is>
-      </c>
-      <c r="M10" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  李宁子2017/9/10</t>
-        </is>
-      </c>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="14" t="n"/>
+      <c r="M10" s="14" t="n"/>
       <c r="N10" s="14" t="n"/>
       <c r="O10" s="14" t="n"/>
       <c r="P10" s="14" t="n"/>

</xml_diff>